<commit_message>
Added Excel Sales Dashboard project
</commit_message>
<xml_diff>
--- a/Pi-vote tables.xlsx
+++ b/Pi-vote tables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Documents\excel.xml\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BEB4DB0-98EB-47EC-8B18-01FBCD56C1EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DB67A16-3B96-4821-A4E9-D34D5F17050F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="5" xr2:uid="{677CDC1A-40C3-45B3-A91A-2C9695995AB5}"/>
   </bookViews>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="607" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="257">
   <si>
     <t>Region</t>
   </si>
@@ -993,6 +993,9 @@
   </si>
   <si>
     <t>Highest no of Units</t>
+  </si>
+  <si>
+    <t>S</t>
   </si>
 </sst>
 </file>
@@ -24246,7 +24249,7 @@
         <v>10</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>19</v>
+        <v>256</v>
       </c>
       <c r="D13" s="2">
         <v>10</v>
@@ -24376,7 +24379,11 @@
         <v>249</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="16.2" customHeight="1"/>
+    <row r="8" spans="1:7" ht="16.2" customHeight="1">
+      <c r="A8" t="s">
+        <v>256</v>
+      </c>
+    </row>
     <row r="11" spans="1:7" ht="25.8">
       <c r="A11" s="63"/>
       <c r="B11" s="64"/>

</xml_diff>